<commit_message>
UPDATE THE COMPILER CHECKS, TESTS AND DOC VERSIONS AND HOPE IT WORKS THIS TIME!
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -1,35 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schema data_product" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Support" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SLA" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Servers" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fundamentals" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schema data_product" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Relationships" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Quality" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Support" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Team" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Roles" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SLA" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Servers" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Pricing" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Custom Properties" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="DET Models" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DET Model Inputs" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="DET Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="DET Source Schema" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="DET Mapping" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="DET Parameters" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="DET Relationships" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Operational Validation" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Operational Parameters" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="DET Lookups" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="DET Build" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="_DET Lists" sheetId="24" state="veryHidden" r:id="rId24"/>
+    <sheet name="_DET Metadata" sheetId="25" state="veryHidden" r:id="rId25"/>
+    <sheet name="_DET Context" sheetId="26" state="veryHidden" r:id="rId26"/>
+    <sheet name="_DET Raw ODCS" sheetId="27" state="veryHidden" r:id="rId27"/>
   </sheets>
   <definedNames>
     <definedName name="apiVersion">Fundamentals!$C$5</definedName>
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v2.3.0</t>
+          <t>v3.0.6</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>2.3.0</t>
+          <t>3.0.6</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 3.0.6 -> 3.0.7
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v3.0.6</t>
+          <t>v3.0.7</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>3.0.6</t>
+          <t>3.0.7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 3.0.7 -> 3.1.0
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v3.0.7</t>
+          <t>v3.1.0</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>3.0.7</t>
+          <t>3.1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 3.1.0 -> 3.2.0
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v3.1.0</t>
+          <t>v3.2.0</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>3.1.0</t>
+          <t>3.2.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 3.2.0 -> 4.0.0
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v3.2.0</t>
+          <t>v4.0.0</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>3.2.0</t>
+          <t>4.0.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 4.0.0 -> 4.0.1
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v4.0.0</t>
+          <t>v4.0.1</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>4.0.0</t>
+          <t>4.0.1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 4.0.1 -> 4.0.2
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v4.0.1</t>
+          <t>v4.0.2</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>4.0.1</t>
+          <t>4.0.2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 4.0.2 -> 4.0.3
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v4.0.2</t>
+          <t>v4.0.3</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>4.0.2</t>
+          <t>4.0.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 4.0.3 -> 4.1.0
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v4.0.3</t>
+          <t>v4.1.0</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>4.0.3</t>
+          <t>4.1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
bump version 4.1.0 -> 4.1.1
</commit_message>
<xml_diff>
--- a/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
+++ b/python/src/dbt_data_engineering_toolkit_compiler/resources/data_product.xlsx
@@ -13444,7 +13444,7 @@
       </c>
       <c r="B8" s="166" t="inlineStr">
         <is>
-          <t>v4.1.0</t>
+          <t>v4.1.1</t>
         </is>
       </c>
       <c r="C8" s="152" t="inlineStr">
@@ -14375,7 +14375,7 @@
       </c>
       <c r="B4" s="152" t="inlineStr">
         <is>
-          <t>4.1.0</t>
+          <t>4.1.1</t>
         </is>
       </c>
     </row>

</xml_diff>